<commit_message>
Updated smoke test runs
</commit_message>
<xml_diff>
--- a/docs/customer-frontend-qa-checklist-dev-smoke-env.xlsx
+++ b/docs/customer-frontend-qa-checklist-dev-smoke-env.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayanc\OneDrive\Desktop\cabbo-frontends\cabbo-customer-frontend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B39AC99-5995-4155-9A4D-D9F53DDCBE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAC6143-92D4-4907-9372-C4E652115AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="168">
   <si>
     <t>Cabbo Customer Frontend QA Checklist (Dev Smoke Env)</t>
   </si>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="B9">
         <f>COUNTIF(Checklist!H2:H200,"Pass")</f>
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12">
         <f>COUNTIF(Checklist!H2:H200,"")</f>
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1945,7 +1945,9 @@
       <c r="G18" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H18" s="9"/>
+      <c r="H18" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I18" s="6" t="s">
         <v>166</v>
       </c>
@@ -1979,7 +1981,9 @@
       <c r="G19" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="H19" s="9"/>
+      <c r="H19" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I19" s="6" t="s">
         <v>166</v>
       </c>
@@ -2013,7 +2017,9 @@
       <c r="G20" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="H20" s="9"/>
+      <c r="H20" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I20" s="6" t="s">
         <v>166</v>
       </c>
@@ -2047,7 +2053,9 @@
       <c r="G21" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="H21" s="9"/>
+      <c r="H21" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I21" s="6" t="s">
         <v>166</v>
       </c>
@@ -2081,7 +2089,9 @@
       <c r="G22" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H22" s="9"/>
+      <c r="H22" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I22" s="6" t="s">
         <v>166</v>
       </c>
@@ -2149,7 +2159,9 @@
       <c r="G24" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="H24" s="9"/>
+      <c r="H24" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I24" s="6" t="s">
         <v>166</v>
       </c>
@@ -2183,7 +2195,9 @@
       <c r="G25" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="H25" s="9"/>
+      <c r="H25" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I25" s="6" t="s">
         <v>166</v>
       </c>
@@ -2217,7 +2231,9 @@
       <c r="G26" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="H26" s="9"/>
+      <c r="H26" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I26" s="6" t="s">
         <v>166</v>
       </c>
@@ -2251,7 +2267,9 @@
       <c r="G27" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="H27" s="9"/>
+      <c r="H27" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I27" s="6" t="s">
         <v>166</v>
       </c>
@@ -2319,7 +2337,9 @@
       <c r="G29" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="H29" s="9"/>
+      <c r="H29" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I29" s="6" t="s">
         <v>166</v>
       </c>
@@ -2353,7 +2373,9 @@
       <c r="G30" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="H30" s="9"/>
+      <c r="H30" s="7" t="s">
+        <v>165</v>
+      </c>
       <c r="I30" s="6" t="s">
         <v>166</v>
       </c>

</xml_diff>